<commit_message>
New height table values ​​corrected
New height table values ​​corrected from the algorithm in v1.0.12
</commit_message>
<xml_diff>
--- a/AdditionalData/Tables/Courses just before changes in thickness thickness.xlsx
+++ b/AdditionalData/Tables/Courses just before changes in thickness thickness.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="me refiero a dividir por 0.71 y" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -166,16 +166,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -372,375 +376,375 @@
   <dimension ref="A1:AA18"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="n">
+      <c r="C1" s="3" t="n">
         <v>45663</v>
       </c>
-      <c r="D1" s="2" t="n">
+      <c r="D1" s="3" t="n">
         <v>45694</v>
       </c>
-      <c r="E1" s="2" t="n">
+      <c r="E1" s="3" t="n">
         <v>45722</v>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="F1" s="3" t="n">
         <v>45753</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="3" t="n">
         <v>45783</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="H1" s="3" t="n">
         <v>45814</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="I1" s="3" t="n">
         <v>45844</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="3" t="n">
         <v>45875</v>
       </c>
-      <c r="K1" s="2" t="n">
+      <c r="K1" s="3" t="n">
         <v>45906</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="2" t="n">
+      <c r="M1" s="3" t="n">
         <v>45664</v>
       </c>
-      <c r="N1" s="2" t="n">
+      <c r="N1" s="3" t="n">
         <v>45695</v>
       </c>
-      <c r="O1" s="2" t="n">
+      <c r="O1" s="3" t="n">
         <v>45723</v>
       </c>
-      <c r="P1" s="2" t="n">
+      <c r="P1" s="3" t="n">
         <v>45754</v>
       </c>
-      <c r="Q1" s="2" t="n">
+      <c r="Q1" s="3" t="n">
         <v>45784</v>
       </c>
-      <c r="R1" s="2" t="n">
+      <c r="R1" s="3" t="n">
         <v>45815</v>
       </c>
-      <c r="S1" s="2" t="n">
+      <c r="S1" s="3" t="n">
         <v>45845</v>
       </c>
-      <c r="T1" s="2" t="n">
+      <c r="T1" s="3" t="n">
         <v>45876</v>
       </c>
-      <c r="U1" s="2" t="n">
+      <c r="U1" s="3" t="n">
         <v>45907</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="W1" s="2" t="n">
+      <c r="W1" s="3" t="n">
         <v>45665</v>
       </c>
-      <c r="X1" s="2" t="n">
+      <c r="X1" s="3" t="n">
         <v>45696</v>
       </c>
-      <c r="Y1" s="2" t="n">
+      <c r="Y1" s="3" t="n">
         <v>45724</v>
       </c>
-      <c r="Z1" s="2" t="n">
+      <c r="Z1" s="3" t="n">
         <v>45755</v>
       </c>
-      <c r="AA1" s="2" t="n">
+      <c r="AA1" s="3" t="n">
         <v>45785</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="P4" s="1" t="n">
+      <c r="P4" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="Q4" s="1" t="n">
+      <c r="Q4" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="R4" s="1" t="n">
+      <c r="R4" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="S4" s="1" t="n">
+      <c r="S4" s="2" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="T7" s="1" t="n">
+      <c r="T7" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="U7" s="1" t="n">
+      <c r="U7" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="V7" s="1" t="n">
+      <c r="V7" s="2" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="2" t="n">
         <v>82</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="P9" s="1" t="n">
+      <c r="P9" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="Q9" s="1" t="n">
+      <c r="Q9" s="2" t="n">
         <v>97</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>104</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="G10" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="W10" s="1" t="n">
+      <c r="W10" s="2" t="n">
         <v>104</v>
       </c>
-      <c r="X10" s="1" t="n">
+      <c r="X10" s="2" t="n">
         <v>105</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>115</v>
       </c>
-      <c r="O11" s="1" t="n">
+      <c r="O11" s="2" t="n">
         <v>115</v>
       </c>
-      <c r="P11" s="1" t="n">
+      <c r="P11" s="2" t="n">
         <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>124</v>
       </c>
-      <c r="K12" s="1" t="n">
+      <c r="K12" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="V12" s="1" t="n">
+      <c r="V12" s="2" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>134</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="2" t="n">
         <v>136</v>
       </c>
-      <c r="Q13" s="1" t="n">
+      <c r="Q13" s="2" t="n">
         <v>135</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>141</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>142</v>
       </c>
-      <c r="L14" s="1" t="n">
+      <c r="L14" s="2" t="n">
         <v>142</v>
       </c>
-      <c r="V14" s="1" t="n">
+      <c r="V14" s="2" t="n">
         <v>143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>146</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G15" s="2" t="n">
         <v>147</v>
       </c>
-      <c r="P15" s="1" t="n">
+      <c r="P15" s="2" t="n">
         <v>147</v>
       </c>
-      <c r="X15" s="1" t="n">
+      <c r="X15" s="2" t="n">
         <v>146</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>152</v>
       </c>
-      <c r="K16" s="1" t="n">
+      <c r="K16" s="2" t="n">
         <v>152</v>
       </c>
-      <c r="S16" s="1" t="n">
+      <c r="S16" s="2" t="n">
         <v>152</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="1" t="n">
+      <c r="K17" s="2" t="n">
         <v>174</v>
       </c>
-      <c r="L17" s="1" t="n">
+      <c r="L17" s="2" t="n">
         <v>176</v>
       </c>
-      <c r="P17" s="1" t="n">
+      <c r="P17" s="2" t="n">
         <v>175</v>
       </c>
-      <c r="T17" s="1" t="n">
+      <c r="T17" s="2" t="n">
         <v>174</v>
       </c>
-      <c r="U17" s="1" t="n">
+      <c r="U17" s="2" t="n">
         <v>176</v>
       </c>
-      <c r="Y17" s="1" t="n">
+      <c r="Y17" s="2" t="n">
         <v>175</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="1" t="n">
+      <c r="I18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K18" s="1" t="n">
+      <c r="K18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L18" s="1" t="n">
+      <c r="L18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M18" s="1" t="n">
+      <c r="M18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="1" t="n">
+      <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O18" s="1" t="n">
+      <c r="O18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P18" s="1" t="n">
+      <c r="P18" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="Q18" s="1" t="n">
+      <c r="Q18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="R18" s="1" t="n">
+      <c r="R18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="1" t="n">
+      <c r="S18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="T18" s="1" t="n">
+      <c r="T18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U18" s="1" t="n">
+      <c r="U18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V18" s="1" t="n">
+      <c r="V18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="W18" s="1" t="n">
+      <c r="W18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="X18" s="1" t="n">
+      <c r="X18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="Y18" s="1" t="n">
+      <c r="Y18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Z18" s="1" t="n">
+      <c r="Z18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="1" t="n">
+      <c r="AA18" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>